<commit_message>
added ToC, new exercise, and new frontpage fig
</commit_message>
<xml_diff>
--- a/output/CD-3_dados_pesquisa_opiniao_produto.xlsx
+++ b/output/CD-3_dados_pesquisa_opiniao_produto.xlsx
@@ -401,7 +401,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -409,7 +409,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -417,7 +417,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -425,7 +425,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
reestruturação da apresentação e revisão geral
</commit_message>
<xml_diff>
--- a/output/CD-3_dados_pesquisa_opiniao_produto.xlsx
+++ b/output/CD-3_dados_pesquisa_opiniao_produto.xlsx
@@ -430,42 +430,42 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>